<commit_message>
1.1 (31): swim pace as Garmin shows it
The pace filled in from Apple Health divided the WHOLE workout by the
distance, so a pool session's rest at the wall counted as swimming: his
1:56 swim of 21 September came out as 3:39 and was saved into the plan.
Now the swimming time only — the union of the swim-distance samples the same
app wrote inside the workout, else the watch's laps or segments, else the
workout minus its pauses; the whole workout only when none of those exist.

UI test #5 opens a swim, uses the pretend Garmin pool swim (46.5 min in all,
1,275 m, 24.7 min swimming) and expects 1:56 — red with 3:39 when the old
rule is put back. The test workbook gains the "Avg Pace/Pwr" column his plan
has, without which the pace box never appears.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UITests/Fixtures/plan.xlsx
+++ b/UITests/Fixtures/plan.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,6 +481,11 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Effort</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Avg Pace/Pwr</t>
         </is>
       </c>
     </row>

</xml_diff>